<commit_message>
update README and uploaded .ris files
</commit_message>
<xml_diff>
--- a/lit_search_output/PRISMA_flow_numbers.xlsx
+++ b/lit_search_output/PRISMA_flow_numbers.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PRISMA Flow Numbers" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,9 +77,21 @@
       <sz val="9.5"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <sz val="11"/>
     </font>
-    <font/>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="16">
     <fill>
@@ -171,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -222,33 +234,39 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -614,31 +632,31 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="4" customWidth="1" style="21" min="1" max="1"/>
-    <col width="46" customWidth="1" style="21" min="2" max="2"/>
-    <col width="12" customWidth="1" style="21" min="3" max="3"/>
-    <col width="42" customWidth="1" style="21" min="4" max="4"/>
+    <col width="4" customWidth="1" style="23" min="1" max="1"/>
+    <col width="46" customWidth="1" style="23" min="2" max="2"/>
+    <col width="12" customWidth="1" style="23" min="3" max="3"/>
+    <col width="42" customWidth="1" style="23" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="21">
-      <c r="A1" s="23" t="inlineStr">
+    <row r="1" ht="30" customHeight="1" s="23">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>PRISMA 2020 Flow Numbers — SocEnRep Literature Search</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="16.05" customHeight="1" s="21">
+    <row r="2" ht="16.05" customHeight="1" s="23">
       <c r="A2" s="28" t="inlineStr">
         <is>
-          <t>Search date: 2026-03-12  |  Source: OpenAlex  |  Tool: ASReview  |  Last updated: 2026-04-01</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1" s="21"/>
-    <row r="4" ht="19.95" customHeight="1" s="21">
+          <t>Search date: 2026-03-12  |  Source: OpenAlex  |  Tool: ASReview  |  Last updated: 2026-05-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1" s="23"/>
+    <row r="4" ht="19.95" customHeight="1" s="23">
       <c r="A4" s="1" t="n"/>
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -656,14 +674,14 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="22.05" customHeight="1" s="21">
+    <row r="5" ht="22.05" customHeight="1" s="23">
       <c r="A5" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  IDENTIFICATION</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="25.2" customHeight="1" s="21">
+    <row r="6" ht="25.2" customHeight="1" s="23">
       <c r="A6" s="2" t="n"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -679,7 +697,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="25.2" customHeight="1" s="21">
+    <row r="7" ht="25.2" customHeight="1" s="23">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -699,7 +717,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="25.2" customHeight="1" s="21">
+    <row r="8" ht="25.2" customHeight="1" s="23">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -719,7 +737,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="21">
+    <row r="9" ht="18" customHeight="1" s="23">
       <c r="A9" s="9" t="n"/>
       <c r="B9" s="10" t="inlineStr">
         <is>
@@ -735,7 +753,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="21">
+    <row r="10" ht="18" customHeight="1" s="23">
       <c r="A10" s="2" t="n"/>
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -751,15 +769,15 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="7.95" customHeight="1" s="21"/>
-    <row r="12" ht="22.05" customHeight="1" s="21">
+    <row r="11" ht="7.95" customHeight="1" s="23"/>
+    <row r="12" ht="22.05" customHeight="1" s="23">
       <c r="A12" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">  SCREENING  (Title &amp; Abstract — ASReview)</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="21">
+    <row r="13" ht="18" customHeight="1" s="23">
       <c r="A13" s="2" t="n"/>
       <c r="B13" s="3" t="inlineStr">
         <is>
@@ -771,7 +789,7 @@
       </c>
       <c r="D13" s="5" t="n"/>
     </row>
-    <row r="14" ht="18" customHeight="1" s="21">
+    <row r="14" ht="18" customHeight="1" s="23">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -791,7 +809,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="21">
+    <row r="15" ht="18" customHeight="1" s="23">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
@@ -811,7 +829,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="21">
+    <row r="16" ht="18" customHeight="1" s="23">
       <c r="A16" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
@@ -831,7 +849,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="25.2" customHeight="1" s="21">
+    <row r="17" ht="25.2" customHeight="1" s="23">
       <c r="A17" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -851,7 +869,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" s="21">
+    <row r="18" ht="18" customHeight="1" s="23">
       <c r="A18" s="9" t="n"/>
       <c r="B18" s="12" t="inlineStr">
         <is>
@@ -867,7 +885,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" s="21">
+    <row r="19" ht="18" customHeight="1" s="23">
       <c r="A19" s="2" t="n"/>
       <c r="B19" s="3" t="inlineStr">
         <is>
@@ -879,8 +897,8 @@
       </c>
       <c r="D19" s="5" t="n"/>
     </row>
-    <row r="20" ht="7.95" customHeight="1" s="21"/>
-    <row r="21" ht="22.05" customHeight="1" s="21">
+    <row r="20" ht="7.95" customHeight="1" s="23"/>
+    <row r="21" ht="22.05" customHeight="1" s="23">
       <c r="A21" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">  ELIGIBILITY  (Full-text Screening)</t>
@@ -899,7 +917,7 @@
       </c>
       <c r="D22" s="5" t="n"/>
     </row>
-    <row r="23" ht="37.8" customHeight="1" s="21">
+    <row r="23" ht="37.8" customHeight="1" s="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -919,7 +937,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="25.2" customHeight="1" s="21">
+    <row r="24" ht="25.2" customHeight="1" s="23">
       <c r="A24" s="9" t="n"/>
       <c r="B24" s="12" t="inlineStr">
         <is>
@@ -935,7 +953,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="25.2" customHeight="1" s="21">
+    <row r="25" ht="25.2" customHeight="1" s="23">
       <c r="A25" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -955,7 +973,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="25.2" customHeight="1" s="21">
+    <row r="26" ht="25.2" customHeight="1" s="23">
       <c r="A26" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -975,7 +993,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="25.2" customHeight="1" s="21">
+    <row r="27" ht="25.2" customHeight="1" s="23">
       <c r="A27" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -995,7 +1013,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="37.8" customHeight="1" s="21">
+    <row r="28" ht="37.8" customHeight="1" s="23">
       <c r="A28" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -1015,7 +1033,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="37.8" customHeight="1" s="21">
+    <row r="29" ht="37.8" customHeight="1" s="23">
       <c r="A29" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -1035,15 +1053,15 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="7.95" customHeight="1" s="21"/>
-    <row r="31" ht="22.05" customHeight="1" s="21">
+    <row r="30" ht="7.95" customHeight="1" s="23"/>
+    <row r="31" ht="22.05" customHeight="1" s="23">
       <c r="A31" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  INCLUDED</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="25.2" customHeight="1" s="21">
+    <row r="32" ht="25.2" customHeight="1" s="23">
       <c r="A32" s="2" t="n"/>
       <c r="B32" s="3" t="inlineStr">
         <is>
@@ -1059,7 +1077,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="25.2" customHeight="1" s="21">
+    <row r="33" ht="25.2" customHeight="1" s="23">
       <c r="A33" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -1079,7 +1097,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="25.2" customHeight="1" s="21">
+    <row r="34" ht="25.2" customHeight="1" s="23">
       <c r="A34" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
@@ -1099,8 +1117,8 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="7.95" customHeight="1" s="21"/>
-    <row r="36" ht="22.05" customHeight="1" s="21">
+    <row r="35" ht="7.95" customHeight="1" s="23"/>
+    <row r="36" ht="22.05" customHeight="1" s="23">
       <c r="A36" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  SNOWBALLING</t>
@@ -1114,7 +1132,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="25.2" customHeight="1" s="21">
+    <row r="39" ht="25.2" customHeight="1" s="23">
       <c r="B39" s="29" t="inlineStr">
         <is>
           <t>Records retrieved (new, after dedup against original pool)</t>
@@ -1123,56 +1141,56 @@
       <c r="C39" s="29" t="n">
         <v>2445</v>
       </c>
-      <c r="D39" s="30" t="inlineStr">
+      <c r="D39" s="21" t="inlineStr">
         <is>
           <t>From 08_forward_snowballing_new.csv; deduplicated against the 5,294-record pool</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="30" t="inlineStr">
+      <c r="A40" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
         </is>
       </c>
-      <c r="B40" s="30" t="inlineStr">
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>Title/abstract screening (ASReview)</t>
         </is>
       </c>
-      <c r="D40" s="30" t="inlineStr">
+      <c r="D40" s="21" t="inlineStr">
         <is>
           <t>09_asreview files; stopping rule = 5% threshold (consecutive irrelevant)</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="7.95" customHeight="1" s="21">
-      <c r="A41" s="30" t="inlineStr">
+    <row r="41" ht="7.95" customHeight="1" s="23">
+      <c r="A41" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
-      <c r="B41" s="30" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  → Labelled relevant</t>
         </is>
       </c>
-      <c r="C41" s="30" t="n">
+      <c r="C41" s="21" t="n">
         <v>18</v>
       </c>
-      <c r="D41" s="30" t="inlineStr">
+      <c r="D41" s="21" t="inlineStr">
         <is>
           <t>Passed to full-text review</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="22.05" customHeight="1" s="21">
-      <c r="A42" s="30" t="inlineStr">
+    <row r="42" ht="22.05" customHeight="1" s="23">
+      <c r="A42" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
-      <c r="B42" s="30" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  → Labelled irrelevant</t>
         </is>
@@ -1181,18 +1199,18 @@
         <v>392</v>
       </c>
     </row>
-    <row r="43" ht="37.8" customHeight="1" s="21">
-      <c r="A43" s="30" t="inlineStr">
+    <row r="43" ht="37.8" customHeight="1" s="23">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">        </t>
         </is>
       </c>
-      <c r="B43" s="30" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  → Not labelled (stopping rule reached)</t>
         </is>
       </c>
-      <c r="C43" s="30" t="n">
+      <c r="C43" s="21" t="n">
         <v>2035</v>
       </c>
     </row>
@@ -1205,7 +1223,7 @@
       <c r="C44" s="29" t="n">
         <v>2427</v>
       </c>
-      <c r="D44" s="30" t="inlineStr">
+      <c r="D44" s="21" t="inlineStr">
         <is>
           <t>392 irrelevant + 2,035 not labelled</t>
         </is>
@@ -1222,22 +1240,22 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="30" t="inlineStr">
+      <c r="A46" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">    </t>
         </is>
       </c>
-      <c r="B46" s="30" t="inlineStr">
+      <c r="B46" s="21" t="inlineStr">
         <is>
           <t>Removed (content unsuitable)</t>
         </is>
       </c>
-      <c r="C46" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="D46" s="30" t="inlineStr">
-        <is>
-          <t>See removed.ris: 3× Banati 2016, Costa 2024, Dudda 2026 — all content unsuitable</t>
+      <c r="C46" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D46" s="33" t="inlineStr">
+        <is>
+          <t>Forward.ris: 18 ASReview-relevant assessed at full-text; 6 removed (content unsuitable), 12 included</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1265,12 @@
           <t>Included from forward snowballing</t>
         </is>
       </c>
-      <c r="C47" s="29" t="n">
-        <v>13</v>
-      </c>
-      <c r="D47" s="30" t="inlineStr">
-        <is>
-          <t>Forward.ris minus removed.ris (18 − 5)</t>
+      <c r="C47" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="D47" s="33" t="inlineStr">
+        <is>
+          <t>Forward.ris (12 records; confirmed against Zotero subcollection)</t>
         </is>
       </c>
     </row>
@@ -1269,12 +1287,12 @@
           <t>Records identified from reference lists of 124 included papers</t>
         </is>
       </c>
-      <c r="C50" s="29" t="n">
+      <c r="C50" s="32" t="n">
         <v>5</v>
       </c>
-      <c r="D50" s="30" t="inlineStr">
-        <is>
-          <t>See Backward.ris: Whitehouse 2019, Knöpfle &amp; Schatto-Eckrodt 2024, Hayden et al. 2023, Vilhuber et al. 2022, Horbach et al. 2026</t>
+      <c r="D50" s="33" t="inlineStr">
+        <is>
+          <t>Backward.ris (5 records): Whitehouse 2019, Horbach et al. 2026, Vilhuber et al. 2022, Hayden et al. 2023, Knöpfle &amp; Schatto-Eckrodt 2024</t>
         </is>
       </c>
     </row>
@@ -1284,168 +1302,286 @@
           <t>Included from backward snowballing</t>
         </is>
       </c>
-      <c r="C51" s="29" t="n">
+      <c r="C51" s="32" t="n">
         <v>5</v>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Grey Literature &amp; Expert Consultation (Step 4c)</t>
+        </is>
+      </c>
+    </row>
     <row r="53">
-      <c r="A53" s="29" t="inlineStr">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    </t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="inlineStr">
+        <is>
+          <t>NBER, IZA DP, OSF preprints (SocArXiv, ArXiv) via OpenAlex</t>
+        </is>
+      </c>
+      <c r="C53" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="33" t="inlineStr">
+        <is>
+          <t>Confirmed already indexed in OpenAlex (2026-04-01); no new records beyond initial pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    </t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="inlineStr">
+        <is>
+          <t>SSOAR GESIS keyword search (“computational reproducibility”)</t>
+        </is>
+      </c>
+      <c r="C54" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D54" s="33" t="inlineStr">
+        <is>
+          <t>Search conducted 2026-04-01; 3 records returned (Schoch et al. 2024; Knöpfle &amp; Schatto-Eckrodt 2024; Weller &amp; Kinder-Kurlanda 2016) — all already included in pool</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        </t>
+        </is>
+      </c>
+      <c r="B55" s="33" t="inlineStr">
+        <is>
+          <t>Snowballed from social media / newsletter</t>
+        </is>
+      </c>
+      <c r="C55" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D55" s="33" t="inlineStr">
+        <is>
+          <t>Miske et al. (2026); Nosek et al. (2025) — Recommendations.ris</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        </t>
+        </is>
+      </c>
+      <c r="B56" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  → Expert referral</t>
+        </is>
+      </c>
+      <c r="C56" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>Bleier, Arnim (2025) — "What is Computational Reproducibility?"; ACRe/BITSS (2022) — "Guide for Accelerating Computational Reproducibility in the Social Sciences" — Recommendations.ris</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>Included from grey literature &amp; expert consultation</t>
+        </is>
+      </c>
+      <c r="C57" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D57" s="33" t="inlineStr">
+        <is>
+          <t>2 (social media/newsletter) + 2 (expert referral)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15.6" customHeight="1" s="23"/>
+    <row r="60">
+      <c r="A60" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  SNOWBALLING TOTAL INCLUDED</t>
         </is>
       </c>
-      <c r="B53" s="29" t="inlineStr"/>
-      <c r="C53" s="29" t="n">
-        <v>18</v>
-      </c>
-      <c r="D53" s="30" t="inlineStr">
-        <is>
-          <t>13 (forward) + 5 (backward)</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="29" t="inlineStr">
+      <c r="B60" s="29" t="n"/>
+      <c r="C60" s="32" t="n">
+        <v>21</v>
+      </c>
+      <c r="D60" s="33" t="inlineStr">
+        <is>
+          <t>12 (forward) + 5 (backward) + 4 (recommendations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="25.2" customHeight="1" s="23"/>
+    <row r="62">
+      <c r="A62" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">  GRAND TOTAL INCLUDED</t>
         </is>
       </c>
-      <c r="B55" s="29" t="inlineStr">
-        <is>
-          <t>(initial search + snowballing)</t>
-        </is>
-      </c>
-      <c r="C55" s="29" t="n">
-        <v>142</v>
-      </c>
-      <c r="D55" s="30" t="inlineStr">
-        <is>
-          <t>124 (initial) + 13 (forward snowballing) + 5 (backward snowballing)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="22" t="inlineStr">
+      <c r="B62" s="32" t="inlineStr">
+        <is>
+          <t>(initial search + snowballing + grey literature)</t>
+        </is>
+      </c>
+      <c r="C62" s="32" t="n">
+        <v>145</v>
+      </c>
+      <c r="D62" s="33" t="inlineStr">
+        <is>
+          <t>124 (initial search) + 12 (forward snowballing) + 5 (backward snowballing) + 4 (recommendations)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  ARITHMETIC CHECKS</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="19" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="2" t="n"/>
+      <c r="B66" s="19" t="inlineStr">
         <is>
           <t>Check 1: Screened = Excluded at T/A + Full-text</t>
         </is>
       </c>
-      <c r="D59" s="5" t="inlineStr">
+      <c r="D66" s="5" t="inlineStr">
         <is>
           <t>5,294 = 5,120 + 174  ✓</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="19" t="inlineStr">
+    <row r="67" ht="15.6" customHeight="1" s="23">
+      <c r="A67" s="2" t="n"/>
+      <c r="B67" s="33" t="inlineStr">
         <is>
           <t>Check 2: Full-text = Not retrieved + Excluded FT + Included</t>
         </is>
       </c>
-      <c r="D60" s="5" t="inlineStr">
+      <c r="D67" s="33" t="inlineStr">
         <is>
           <t>174 = 2 + 48 + 124  ✓</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="19" t="inlineStr">
-        <is>
-          <t>Check 3: File 01 = File 02 + File 03 (direct) + unaccounted</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>174 = 58 + 116 + 0  ✓  (file 02 contains 8 preprint swaps + 2 not found + 48 excluded)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="19" t="inlineStr">
-        <is>
-          <t>Check 4: File 03 total = direct + preprint replacements</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>124 = 116 + 8  ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="30" t="inlineStr">
-        <is>
-          <t>Check 5: Forward snowball total = Relevant + Irrelevant + Not seen</t>
-        </is>
-      </c>
-      <c r="D63" s="30" t="inlineStr">
-        <is>
-          <t>2,445 = 18 + 392 + 2,035  ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="B64" s="30" t="inlineStr">
-        <is>
-          <t>Check 6: Forward FT assessed = Removed + Included</t>
-        </is>
-      </c>
-      <c r="D64" s="30" t="inlineStr">
-        <is>
-          <t>18 = 5 + 13  ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="30" t="inlineStr">
-        <is>
-          <t>Check 7: Grand total = Initial + Forward + Backward</t>
-        </is>
-      </c>
-      <c r="D65" s="30" t="inlineStr">
-        <is>
-          <t>142 = 124 + 13 + 5  ✓</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
+    <row r="68" ht="63" customHeight="1" s="23">
       <c r="A68" s="2" t="n"/>
       <c r="B68" s="19" t="inlineStr">
         <is>
+          <t>Check 3: File 01 = File 02 + File 03 (direct) + unaccounted</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>174 = 58 + 116 + 0  ✓  (file 02 contains 8 preprint swaps + 2 not found + 48 excluded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n"/>
+      <c r="B69" s="19" t="inlineStr">
+        <is>
+          <t>Check 4: File 03 total = direct + preprint replacements</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>124 = 116 + 8  ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="B70" s="21" t="inlineStr">
+        <is>
+          <t>Check 5: Forward snowball total = Relevant + Irrelevant + Not seen</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>2,445 = 18 + 392 + 2,035  ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="B71" s="21" t="inlineStr">
+        <is>
+          <t>Check 6: Forward FT assessed = Removed + Included</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>18 = 6 + 12  ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="21" t="inlineStr">
+        <is>
+          <t>Check 7: Grand total = Initial + Forward + Backward + Recommendations</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>145 = 124 + 12 + 5 + 4  ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="32" t="inlineStr">
+        <is>
+          <t>Check 8: Supplementary total = Forward + Backward + Recommendations</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="inlineStr">
+        <is>
+          <t>21 = 12 + 5 + 4  ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n"/>
+      <c r="B75" s="19" t="inlineStr">
+        <is>
           <t>Next step</t>
         </is>
       </c>
-      <c r="D68" s="17" t="inlineStr">
-        <is>
-          <t>Snowballing complete (2026-03-31 forward, 2026-03-30 backward). Next: grey literature + expert consultation (NBER, IZA DP, SocArXiv, ArXiv, SSOAR, GESIS WP), then PRISMA flow diagram (Step 5 in protocol_logbook.docx).</t>
+      <c r="D75" s="34" t="inlineStr">
+        <is>
+          <t>Grey literature &amp; expert consultation complete (2026-04-02). Snowballing complete (2026-03-31 forward, 2026-03-30 backward). Total corpus: 145 records. Next: PRISMA flow diagram (Step 5 in protocol_logbook.docx) and coding workflow.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A31:D31"/>
+    <mergeCell ref="A74:D74"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A65:D65"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A36:D36"/>
   </mergeCells>

</xml_diff>